<commit_message>
Open maximized, and tell the survey sheet about photos
The window opened at 800x450, the WPF template's default, which nobody had
touched since. The product screen alone now needs about 1100px across for the
photo panel and its two columns of fields, so the first thing anyone did on
launch was drag the window bigger. It starts maximized; the restore size goes
to 1280x800 so dropping out of maximized does not put them back where they
started.

The survey sheet's instructions stopped at step 2. Photos arrive as a folder
rather than a column in the sheet, so somebody reading the sheet had no way to
learn the feature exists. The guide sheet now covers naming pictures after the
barcode, that JPG is required and an iPhone writes HEIC, and that the step can
be repeated or skipped for months and run later.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/initial-stock-survey.xlsx
+++ b/docs/templates/initial-stock-survey.xlsx
@@ -458,6 +458,39 @@
   </x:si>
   <x:si>
     <x:t>so stock does not get doubled. Edit the file and it can be used again.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Photos (optional, step 3)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Product photos are not part of this sheet. They are imported from a FOLDER:</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">   3) press 'Import Photos' and pick the folder of pictures</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name each picture after the product's barcode, the same value you wrote in</x:t>
+  </x:si>
+  <x:si>
+    <x:t>the barcode column:</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">     8801234567890.jpg</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A product with no barcode can use its product_name instead.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Use JPG. A photo taken on an iPhone is HEIC by default and cannot be read -</x:t>
+  </x:si>
+  <x:si>
+    <x:t>set the camera to Most Compatible, or convert the folder to JPG first.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>This step can be repeated as often as you like; photos replace, they do not</x:t>
+  </x:si>
+  <x:si>
+    <x:t>pile up. You can also skip it now and add photos months later.</x:t>
   </x:si>
   <x:si>
     <x:t>dosage_form - allowed values</x:t>
@@ -1203,7 +1236,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A56"/>
+  <x:dimension ref="A1:A72"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="92.710625" style="0" customWidth="1"/>
@@ -1421,57 +1454,132 @@
     </x:row>
     <x:row r="46" spans="1:1">
       <x:c r="A46" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:1">
       <x:c r="A47" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:1">
       <x:c r="A48" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:1">
       <x:c r="A49" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:1">
       <x:c r="A50" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:1">
       <x:c r="A51" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:1">
       <x:c r="A52" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:1">
       <x:c r="A53" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:1">
       <x:c r="A54" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:1">
       <x:c r="A55" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:1">
       <x:c r="A56" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" spans="1:1">
+      <x:c r="A57" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" spans="1:1">
+      <x:c r="A58" s="4" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" spans="1:1">
+      <x:c r="A60" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" spans="1:1">
+      <x:c r="A61" s="0" t="s">
         <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" spans="1:1">
+      <x:c r="A62" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" spans="1:1">
+      <x:c r="A63" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" spans="1:1">
+      <x:c r="A64" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" spans="1:1">
+      <x:c r="A65" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" spans="1:1">
+      <x:c r="A66" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" spans="1:1">
+      <x:c r="A67" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" spans="1:1">
+      <x:c r="A68" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" spans="1:1">
+      <x:c r="A69" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" spans="1:1">
+      <x:c r="A70" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" spans="1:1">
+      <x:c r="A71" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" spans="1:1">
+      <x:c r="A72" s="0" t="s">
+        <x:v>73</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1499,16 +1607,16 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" s="5" customFormat="1">
       <x:c r="A1" s="5" t="s">
-        <x:v>63</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B1" s="5" t="s">
-        <x:v>64</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C1" s="5" t="s">
-        <x:v>65</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D1" s="5" t="s">
-        <x:v>66</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -1516,13 +1624,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
@@ -1530,13 +1638,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
@@ -1544,13 +1652,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
@@ -1558,13 +1666,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
@@ -1572,13 +1680,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
@@ -1586,13 +1694,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
@@ -1600,13 +1708,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:4">
@@ -1614,13 +1722,13 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:4">
@@ -1628,13 +1736,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:4">
@@ -1642,13 +1750,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:4">
@@ -1656,13 +1764,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:4">
@@ -1670,13 +1778,13 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:4">
@@ -1684,13 +1792,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:4">
@@ -1698,13 +1806,13 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:4">
@@ -1712,13 +1820,13 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:4">
@@ -1726,13 +1834,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:4">
@@ -1740,13 +1848,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:4">
@@ -1754,13 +1862,13 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:4">
@@ -1768,13 +1876,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>121</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>